<commit_message>
Cashiering: BDOI's payment files with MFT intake and channel simulator, OR at Disbursement approval, receipt forms and printing, series formats, reports in BDOI's layouts, unapplied list, search log, day-end list and device restriction setting
Payment files of Bills Payment, PDC, CLPC, Trade, Direct Credit and Commission Schedule in BDOI's layouts with name, size, duplicate, header and TOTAL checks, run report, reprocessing and MFT folder intake with the refusal alert.
Settlement ORs kept until Disbursement approves the payment request (setting).
AR and OR forms with versions approved by a second user, certificate numbers, REPRINT mark, copies, ZIP and skip.
Series with year and number format; print queue and re-print search.
Reports named <Report Name>_<MMDDYYYY> with BDOI's columns; summary per disposition.
Unapplied payment list, search log, day-end totals, other income SOA selection, PR 2307 base and device restriction settings.
Coverage workbook, Appendix G and Appendix R updated.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
@@ -1674,7 +1674,7 @@
       <c r="C41" s="12" t="inlineStr"/>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Open, Decided, Withdrawn</t>
+          <t>Open, Configurable – BDOI to confirm the setting, Decided, Withdrawn</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Issue at save for counter, file and PDC payments, so the client gets the AR at once and the series is used in order; give the TL a daily review list. If BDOI keeps the posting step, make it a configurable approval per receipt type (for example manual ORs only). (the system reference FRS: “Issue AR and Apply” issues the AR from the branch series, applies the payment and opens the receipt (FR-OP-011); ORs likewise (FR-OP-012).)</t>
+          <t>Issue at save for counter, file and PDC payments, so the client gets the AR at once and the series is used in order; give the TL a daily review list. If BDOI keeps the posting step, make it a configurable approval per receipt type (for example manual ORs only). (the system reference FRS: “Issue AR and Apply” issues the AR from the branch series, applies the payment and opens the receipt (FR-OP-011); ORs likewise (FR-OP-012).) Available as a setting: Setting of the receipts that need the posting step: AR and OR (BDOI's reading) by default; blank issues the number at save.</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4195,7 +4195,7 @@
       <c r="I5" s="12" t="inlineStr"/>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4217,7 +4217,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Both, under one Reinstate action with the BRD's reasons: “Due to Cancellation” and bounced check restore a cancelled receipt; mis-application and withholding tax adjustment reverse the application of an issued receipt for re-application. (the system reference FRS: Reinstate a cancelled receipt in full or in part; the reinstated amount is applied to the encoded invoice (FR-OP-014). Reversal of an issued receipt's application is the payment reversal of Incoming Requests.)</t>
+          <t>Both, under one Reinstate action with the BRD's reasons: “Due to Cancellation” and bounced check restore a cancelled receipt; mis-application and withholding tax adjustment reverse the application of an issued receipt for re-application. (the system reference FRS: Reinstate a cancelled receipt in full or in part; the reinstated amount is applied to the encoded invoice (FR-OP-014). Reversal of an issued receipt's application is the payment reversal of Incoming Requests.) Available as a setting: Setting of what Reinstate does: issued receipts (BDOI's reading), cancelled receipts, or both (by default).</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -4231,7 +4231,7 @@
       <c r="I6" s="12" t="inlineStr"/>
       <c r="J6" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's prefixes with the year (for example CN-AR-2026-000001); the numbering is configuration. (the system reference FRS: Cancellation CAN-yyyy-n and reinstatement RIN-yyyy-n (FR-OP-013, 014).)</t>
+          <t>Adopt BDOI's prefixes with the year (for example CN-AR-2026-000001); the numbering is configuration. (the system reference FRS: Cancellation CAN-yyyy-n and reinstatement RIN-yyyy-n (FR-OP-013, 014).) Available as a setting: Setting of the record number format: prefix, type and sequence by default.</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -4267,7 +4267,7 @@
       <c r="I7" s="12" t="inlineStr"/>
       <c r="J7" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Keep 10.00 as in the BRD unless BDOI decides otherwise; it is a parameter. (the system reference FRS: Default 10.00 for premium and excess, configurable (FR-OP-023).)</t>
+          <t>Keep 10.00 as in the BRD unless BDOI decides otherwise; it is a parameter. (the system reference FRS: Default 10.00 for premium and excess, configurable (FR-OP-023).) Available as a setting: Setting of the minimal balance threshold: 10.00 by default (BRD).</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -4303,7 +4303,7 @@
       <c r="I8" s="12" t="inlineStr"/>
       <c r="J8" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4325,7 +4325,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Keep FST as its own component after LGT (it is booked on fire policies); apply check payments before cash payments on the same invoice on the same day. (the system reference FRS: DST, VAT, LGT, FST, other charges, basic premium; check before cash open (FR-OP-019, OQ09).)</t>
+          <t>Keep FST as its own component after LGT (it is booked on fire policies); apply check payments before cash payments on the same invoice on the same day. (the system reference FRS: DST, VAT, LGT, FST, other charges, basic premium; check before cash open (FR-OP-019, OQ09).) Available as a setting: Setting of the order of the payments of one posting run: checks before cash by default.</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -4339,7 +4339,7 @@
       <c r="I9" s="12" t="inlineStr"/>
       <c r="J9" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4361,7 +4361,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Accept the check when it is presented (a post-dated check goes to the PDC warehouse); keep the holding period for remittance only. (the system reference FRS: No check-date validation at receipt; 3 banking days before the payment is remitted (FR-OP-031, RMTID.017).)</t>
+          <t>Accept the check when it is presented (a post-dated check goes to the PDC warehouse); keep the holding period for remittance only. (the system reference FRS: No check-date validation at receipt; 3 banking days before the payment is remitted (FR-OP-031, RMTID.017).) Available as a setting: Settings of the check date rule (on) and of the holding period (4 working days).</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -4375,7 +4375,7 @@
       <c r="I10" s="12" t="inlineStr"/>
       <c r="J10" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's reading: the file identifies unmatched payments already receipted, so no second AR; new money arrives through the other channels. (the system reference FRS: Every Direct Credit row is a new payment with its own AR (FR-OP-015).)</t>
+          <t>Adopt BDOI's reading: the file identifies unmatched payments already receipted, so no second AR; new money arrives through the other channels. (the system reference FRS: Every Direct Credit row is a new payment with its own AR (FR-OP-015).) Available as a setting: Setting of the reading of the Direct Credit file: identification of payments already received (BDOI's reading) by default.</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -4411,7 +4411,7 @@
       <c r="I11" s="12" t="inlineStr"/>
       <c r="J11" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's rule; it matches how our Adjustment FRs handle remitted premium (AR Insurer, FR-OP-057). (the system reference FRS: Every application is reversed and the invoices are outstanding again (FR-OP-013).)</t>
+          <t>Adopt BDOI's rule; it matches how our Adjustment FRs handle remitted premium (AR Insurer, FR-OP-057). (the system reference FRS: Every application is reversed and the invoices are outstanding again (FR-OP-013).) Available as a setting: Setting of the cancellation of a remitted AR: AR insurer refund (BDOI's reading) by default.</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -4447,7 +4447,7 @@
       <c r="I12" s="12" t="inlineStr"/>
       <c r="J12" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4469,7 +4469,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Line-level processing as BRQID.006 asks, with the exceptions listed; partial payments allowed and shown as such. (the system reference FRS: Valid lines are staged and issued; failed lines stay staged with their reason (FR-OP-021).)</t>
+          <t>Line-level processing as BRQID.006 asks, with the exceptions listed; partial payments allowed and shown as such. (the system reference FRS: Valid lines are staged and issued; failed lines stay staged with their reason (FR-OP-021).) Available as a setting: Setting of the commission schedule with failed or unmatched lines: valid lines processed (BRD) by default; whole file refused available.</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -4483,7 +4483,7 @@
       <c r="I13" s="12" t="inlineStr"/>
       <c r="J13" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4541,7 +4541,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Comptrollership decides the point at which the commission OR is issued; moving it to the Disbursement approval is a change to the system. (the system reference FRS: The commission OR is issued when the Remittance TL approves the batch (FR-OP-035).)</t>
+          <t>Comptrollership decides the point at which the commission OR is issued; moving it to the Disbursement approval is a change to the system. (the system reference FRS: The commission OR is issued when the Remittance TL approves the batch (FR-OP-035).) Available as a setting: Setting of the point the settlement OR is issued: at the approval of Disbursement (BDOI's reading) by default; at the remittance approval available.</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -4555,7 +4555,7 @@
       <c r="I15" s="12" t="inlineStr"/>
       <c r="J15" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4577,7 @@
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Keep Cashiering ownership with requests from Collections, as the BRD-4 Collections FRS specifies; give Marketing read access to the items of its unit. (the system reference FRS: The Cashier assigns and the Cashiering TL approves; Collections asks through Incoming Requests (FR-OP-022; BRD-4).)</t>
+          <t>Keep Cashiering ownership with requests from Collections, as the BRD-4 Collections FRS specifies; give Marketing read access to the items of its unit. (the system reference FRS: The Cashier assigns and the Cashiering TL approves; Collections asks through Incoming Requests (FR-OP-022; BRD-4).) Available as a setting: Setting of what Marketing users see in the unapplied payment list: their marketing unit (BDOI's reading) by default.</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -4591,7 +4591,7 @@
       <c r="I16" s="12" t="inlineStr"/>
       <c r="J16" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Set 50 MB. (the system reference FRS: Not stated; the system accepts files up to 25 MB.)</t>
+          <t>Set 50 MB. (the system reference FRS: Not stated; the system accepts files up to 25 MB.) Available as a setting: Size limit per payment file type: 50 MB by default.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -4735,7 +4735,7 @@
       <c r="I20" s="12" t="inlineStr"/>
       <c r="J20" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4793,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Keep the BRD list (it is a maintained list); add the check-payment restriction if BDOI wants it. (the system reference FRS: The BRD lists in four groups, including Check not picked-up, Negative VAT, Discount not applied, PDC retrieval / replacement, Bounced or returned check, Error printing.)</t>
+          <t>Keep the BRD list (it is a maintained list); add the check-payment restriction if BDOI wants it. (the system reference FRS: The BRD lists in four groups, including Check not picked-up, Negative VAT, Discount not applied, PDC retrieval / replacement, Bounced or returned check, Error printing.) Available as a setting: List of the cancellation reasons allowed for a check payment, by default.</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -4807,7 +4807,7 @@
       <c r="I22" s="12" t="inlineStr"/>
       <c r="J22" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Enforce it through BDO's network and device policy if required; no change to the screens. (the system reference FRS: Log-in from a browser; responsive screens.)</t>
+          <t>Enforce it through BDO's network and device policy if required; no change to the screens. (the system reference FRS: Log-in from a browser; responsive screens.) Available as a setting: Setting of the device restriction: off by default for SIT; on with the company networks and the device header of BDOI IT.</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -4915,7 +4915,7 @@
       <c r="I25" s="12" t="inlineStr"/>
       <c r="J25" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4937,7 +4937,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Bank account mandatory (defaulted by currency as BDOI proposes); remarks optional. (the system reference FRS: Neither field exists on Receive Payment.)</t>
+          <t>Bank account mandatory (defaulted by currency as BDOI proposes); remarks optional. (the system reference FRS: Neither field exists on Receive Payment.) Available as a setting: Setting of the remarks of an AR: mandatory by default.</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -4951,7 +4951,7 @@
       <c r="I26" s="12" t="inlineStr"/>
       <c r="J26" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4973,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Tag per account, defaulted from the client; Comptrollership states the base of the 2% (basic or gross premium); the system keeps the share applied as a parameter. (the system reference FRS: 2% CWT client flag; 98% of the premium applied (FR-OP-018; OQ10).)</t>
+          <t>Tag per account, defaulted from the client; Comptrollership states the base of the 2% (basic or gross premium); the system keeps the share applied as a parameter. (the system reference FRS: 2% CWT client flag; 98% of the premium applied (FR-OP-018; OQ10).) Available as a setting: Setting of the base of the PR 2307: the premium amount by default; the basic premium available.</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -4987,7 +4987,7 @@
       <c r="I27" s="12" t="inlineStr"/>
       <c r="J27" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>BDOI to give one format per receipt kind; the system sets it as the series prefix and range without a change.</t>
+          <t>BDOI to give one format per receipt kind; the system sets it as the series prefix and range without a change. Available as a setting: Settings of the AR and OR number format (prefix, year, branch indicator, sequence) and of the certificate number (AC, branch, month and year, sequence).</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -5095,7 +5095,7 @@
       <c r="I30" s="12" t="inlineStr"/>
       <c r="J30" s="25" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -7168,7 +7168,7 @@
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="J5:J587" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
-      <formula1>'Lists'!$D$2:$D$4</formula1>
+      <formula1>'Lists'!$D$2:$D$5</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="1"/>
@@ -7197,7 +7197,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7262,7 +7262,7 @@
       </c>
       <c r="D3" s="34" t="inlineStr">
         <is>
-          <t>Decided</t>
+          <t>Configurable – BDOI to confirm the setting</t>
         </is>
       </c>
     </row>
@@ -7284,7 +7284,7 @@
       </c>
       <c r="D4" s="34" t="inlineStr">
         <is>
-          <t>Withdrawn</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -7297,6 +7297,11 @@
       <c r="C5" s="34" t="inlineStr">
         <is>
           <t>Approved</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Withdrawn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BDOI-format FRS as the final document: Cashiering v3.2 aligned with BIBS (Create AR/OR, Cashiering Record, Posting, Payment Files, AR and OR Forms, Day-End List, Search Log, Unapplied Payment List and Settlement ORs screens, updated dashboard, receipts, batch print and series screens, settings for the points BDOI decides, integrations, menus and test cases); references to the earlier FRS removed from the Cashiering, User Access Maintenance and Product Maintenance documents and workbooks, traceability from BRD ID to FR item and test cases, table of contents written into the documents, tables fitted with repeated header rows, uniform screenshots and diagrams at 240 dpi
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
@@ -851,7 +851,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>9 October 2026</t>
+          <t>10 October 2026</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2244,7 @@
       <c r="S6" s="12" t="inlineStr"/>
       <c r="T6" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.02.01.02-AC01, TC-FRS-CSH.02.01.02-AC02, TC-FRS-CSH.02.01.02-AC03, TC-FRS-CSH.02.01.02-AC04, TC-OP-011.1-01</t>
+          <t>TC-FRS-CSH.02.01.02-AC01, TC-FRS-CSH.02.01.02-AC02, TC-FRS-CSH.02.01.02-AC03, TC-FRS-CSH.02.01.02-AC04, TC-OP-011.4-01</t>
         </is>
       </c>
     </row>
@@ -2416,7 +2416,7 @@
       <c r="S8" s="12" t="inlineStr"/>
       <c r="T8" s="12" t="inlineStr">
         <is>
-          <t>TC-OP-015.1-01, TC-OP-015.2-01, TC-OP-015.3-01, TC-OP-015.3-02</t>
+          <t>TC-OP-015.4-01, TC-OP-015.4-02, TC-OP-015.1-01, TC-OP-015.2-01, TC-OP-015.3-01</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
       <c r="S11" s="12" t="inlineStr"/>
       <c r="T11" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.07.01.01-AC01, TC-OP-021.1-01, TC-OP-021.1-02, TC-OP-021.2-01, TC-OP-021.2-02</t>
+          <t>TC-FRS-CSH.07.01.01-AC01, TC-OP-021.3-01, TC-OP-021.1-01, TC-OP-021.1-02, TC-OP-021.2-01</t>
         </is>
       </c>
     </row>
@@ -2760,7 +2760,7 @@
       <c r="S12" s="12" t="inlineStr"/>
       <c r="T12" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.05.01.04-AC01, TC-FRS-CSH.05.01.04-AC02, TC-OP-015.1-01, TC-OP-015.2-01, TC-OP-015.3-01</t>
+          <t>TC-FRS-CSH.05.01.04-AC01, TC-FRS-CSH.05.01.04-AC02, TC-OP-015.4-01, TC-OP-015.4-02, TC-OP-015.1-01</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       <c r="S14" s="12" t="inlineStr"/>
       <c r="T14" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.02.04.07-AC01, TC-OP-025.1-01, TC-OP-025.2-01, TC-OP-025.2-02</t>
+          <t>TC-FRS-CSH.02.04.07-AC01, TC-OP-025.3-01, TC-OP-025.3-02, TC-OP-025.1-01, TC-OP-025.2-01</t>
         </is>
       </c>
     </row>
@@ -3018,7 +3018,7 @@
       <c r="S15" s="12" t="inlineStr"/>
       <c r="T15" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.02.06.01-AC01, TC-OP-025.1-01, TC-OP-025.2-01, TC-OP-025.2-02, TC-FRS-CSH.02.06.02-AC01</t>
+          <t>TC-FRS-CSH.02.06.01-AC01, TC-OP-025.3-01, TC-OP-025.3-02, TC-OP-025.1-01, TC-OP-025.2-01</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       <c r="S17" s="12" t="inlineStr"/>
       <c r="T17" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.01.03.02-AC01, TC-FRS-CSH.01.03.02-AC02, TC-FRS-CSH.01.03.02-AC03, TC-OP-003.1-01, TC-OP-003.2-01</t>
+          <t>TC-FRS-CSH.01.03.02-AC01, TC-FRS-CSH.01.03.02-AC02, TC-FRS-CSH.01.03.02-AC03, TC-OP-003.4-01, TC-OP-003.1-01</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
       <c r="S18" s="12" t="inlineStr"/>
       <c r="T18" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.02.04.07-AC01, TC-OP-025.1-01, TC-OP-025.2-01, TC-OP-025.2-02</t>
+          <t>TC-FRS-CSH.02.04.07-AC01, TC-OP-025.3-01, TC-OP-025.3-02, TC-OP-025.1-01, TC-OP-025.2-01</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       <c r="S19" s="12" t="inlineStr"/>
       <c r="T19" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.02.01.16-AC01, TC-OP-011.1-01, TC-OP-011.2-01, TC-OP-011.2-02, TC-OP-011.3-01</t>
+          <t>TC-FRS-CSH.02.01.16-AC01, TC-OP-011.4-01, TC-OP-011.4-02, TC-OP-011.4-03, TC-OP-011.4-04</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       <c r="S20" s="12" t="inlineStr"/>
       <c r="T20" s="12" t="inlineStr">
         <is>
-          <t>TC-FRS-CSH.06.02.02-AC01, TC-FRS-CSH.06.02.02-AC02, TC-OP-022.1-01, TC-OP-022.2-01, TC-OP-022.2-02</t>
+          <t>TC-FRS-CSH.06.02.02-AC01, TC-FRS-CSH.06.02.02-AC02, TC-OP-022.4-01, TC-OP-022.1-01, TC-OP-022.2-01</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>Issue at save for counter, file and PDC payments, so the client gets the AR at once and the series is used in order; give the TL a daily review list. If BDOI keeps the posting step, make it a configurable approval per receipt type (for example manual ORs only). (the system reference FRS: “Issue AR and Apply” issues the AR from the branch series, applies the payment and opens the receipt (FR-OP-011); ORs likewise (FR-OP-012).) Available as a setting: Setting of the receipts that need the posting step: AR and OR (BDOI's reading) by default; blank issues the number at save.</t>
+          <t>Issue at save for counter, file and PDC payments, so the client gets the AR at once and the series is used in order; give the TL a daily review list. If BDOI keeps the posting step, make it a configurable approval per receipt type (for example manual ORs only). Proposed behaviour: “Issue AR and Apply” issues the AR from the branch series, applies the payment and opens the receipt; ORs likewise. Available as a setting: Setting of the receipts that need the posting step: AR and OR (BDOI's reading) by default; blank issues the number at save.</t>
         </is>
       </c>
       <c r="E5" s="12" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>Both, under one Reinstate action with the BRD's reasons: “Due to Cancellation” and bounced check restore a cancelled receipt; mis-application and withholding tax adjustment reverse the application of an issued receipt for re-application. (the system reference FRS: Reinstate a cancelled receipt in full or in part; the reinstated amount is applied to the encoded invoice (FR-OP-014). Reversal of an issued receipt's application is the payment reversal of Incoming Requests.) Available as a setting: Setting of what Reinstate does: issued receipts (BDOI's reading), cancelled receipts, or both (by default).</t>
+          <t>Both, under one Reinstate action with the BRD's reasons: “Due to Cancellation” and bounced check restore a cancelled receipt; mis-application and withholding tax adjustment reverse the application of an issued receipt for re-application. Proposed behaviour: Reinstate a cancelled receipt in full or in part; the reinstated amount is applied to the encoded invoice. Reversal of an issued receipt's application is the payment reversal of Incoming Requests. Available as a setting: Setting of what Reinstate does: issued receipts (BDOI's reading), cancelled receipts, or both (by default).</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's prefixes with the year (for example CN-AR-2026-000001); the numbering is configuration. (the system reference FRS: Cancellation CAN-yyyy-n and reinstatement RIN-yyyy-n (FR-OP-013, 014).) Available as a setting: Setting of the record number format: prefix, type and sequence by default.</t>
+          <t>Adopt BDOI's prefixes with the year (for example CN-AR-2026-000001); the numbering is configuration. Proposed behaviour: Cancellation CAN-yyyy-n and reinstatement RIN-yyyy-n (014). Available as a setting: Setting of the record number format: prefix, type and sequence by default.</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
@@ -4289,7 +4289,7 @@
       </c>
       <c r="D8" s="12" t="inlineStr">
         <is>
-          <t>Keep 10.00 as in the BRD unless BDOI decides otherwise; it is a parameter. (the system reference FRS: Default 10.00 for premium and excess, configurable (FR-OP-023).) Available as a setting: Setting of the minimal balance threshold: 10.00 by default (BRD).</t>
+          <t>Keep 10.00 as in the BRD unless BDOI decides otherwise; it is a parameter. Proposed behaviour: Default 10.00 for premium and excess, configurable. Available as a setting: Setting of the minimal balance threshold: 10.00 by default (BRD).</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Keep FST as its own component after LGT (it is booked on fire policies); apply check payments before cash payments on the same invoice on the same day. (the system reference FRS: DST, VAT, LGT, FST, other charges, basic premium; check before cash open (FR-OP-019, OQ09).) Available as a setting: Setting of the order of the payments of one posting run: checks before cash by default.</t>
+          <t>Keep FST as its own component after LGT (it is booked on fire policies); apply check payments before cash payments on the same invoice on the same day. Proposed behaviour: DST, VAT, LGT, FST, other charges, basic premium; check before cash open. Available as a setting: Setting of the order of the payments of one posting run: checks before cash by default.</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
-          <t>Accept the check when it is presented (a post-dated check goes to the PDC warehouse); keep the holding period for remittance only. (the system reference FRS: No check-date validation at receipt; 3 banking days before the payment is remitted (FR-OP-031, RMTID.017).) Available as a setting: Settings of the check date rule (on) and of the holding period (4 working days).</t>
+          <t>Accept the check when it is presented (a post-dated check goes to the PDC warehouse); keep the holding period for remittance only. Proposed behaviour: No check-date validation at receipt; 3 banking days before the payment is remitted (RMTID.017). Available as a setting: Settings of the check date rule (on) and of the holding period (4 working days).</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's reading: the file identifies unmatched payments already receipted, so no second AR; new money arrives through the other channels. (the system reference FRS: Every Direct Credit row is a new payment with its own AR (FR-OP-015).) Available as a setting: Setting of the reading of the Direct Credit file: identification of payments already received (BDOI's reading) by default.</t>
+          <t>Adopt BDOI's reading: the file identifies unmatched payments already receipted, so no second AR; new money arrives through the other channels. Proposed behaviour: Every Direct Credit row is a new payment with its own AR. Available as a setting: Setting of the reading of the Direct Credit file: identification of payments already received (BDOI's reading) by default.</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's rule; it matches how our Adjustment FRs handle remitted premium (AR Insurer, FR-OP-057). (the system reference FRS: Every application is reversed and the invoices are outstanding again (FR-OP-013).) Available as a setting: Setting of the cancellation of a remitted AR: AR insurer refund (BDOI's reading) by default.</t>
+          <t>Adopt BDOI's rule; it matches how our Adjustment FRs handle remitted premium (AR Insurer). Proposed behaviour: Every application is reversed and the invoices are outstanding again. Available as a setting: Setting of the cancellation of a remitted AR: AR insurer refund (BDOI's reading) by default.</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Line-level processing as BRQID.006 asks, with the exceptions listed; partial payments allowed and shown as such. (the system reference FRS: Valid lines are staged and issued; failed lines stay staged with their reason (FR-OP-021).) Available as a setting: Setting of the commission schedule with failed or unmatched lines: valid lines processed (BRD) by default; whole file refused available.</t>
+          <t>Line-level processing as BRQID.006 asks, with the exceptions listed; partial payments allowed and shown as such. Proposed behaviour: Valid lines are staged and issued; failed lines stay staged with their reason. Available as a setting: Setting of the commission schedule with failed or unmatched lines: valid lines processed (BRD) by default; whole file refused available.</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -4505,7 +4505,7 @@
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>One OR per insurer / payee and certificate per schedule or batch, as CSHID.007 states. (the system reference FRS: One OR per insurer, certificate and payment for Collection details; one OR per remittance batch (FR-OP-021, OQ49).)</t>
+          <t>One OR per insurer / payee and certificate per schedule or batch, as CSHID.007 states. Proposed behaviour: One OR per insurer, certificate and payment for Collection details; one OR per remittance batch.</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -4541,7 +4541,7 @@
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>Comptrollership decides the point at which the commission OR is issued; moving it to the Disbursement approval is a change to the system. (the system reference FRS: The commission OR is issued when the Remittance TL approves the batch (FR-OP-035).) Available as a setting: Setting of the point the settlement OR is issued: at the approval of Disbursement (BDOI's reading) by default; at the remittance approval available.</t>
+          <t>Comptrollership decides the point at which the commission OR is issued; moving it to the Disbursement approval is a change to the system. Proposed behaviour: The commission OR is issued when the Remittance TL approves the batch. Available as a setting: Setting of the point the settlement OR is issued: at the approval of Disbursement (BDOI's reading) by default; at the remittance approval available.</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
@@ -4577,7 +4577,7 @@
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Keep Cashiering ownership with requests from Collections, as the BRD-4 Collections FRS specifies; give Marketing read access to the items of its unit. (the system reference FRS: The Cashier assigns and the Cashiering TL approves; Collections asks through Incoming Requests (FR-OP-022; BRD-4).) Available as a setting: Setting of what Marketing users see in the unapplied payment list: their marketing unit (BDOI's reading) by default.</t>
+          <t>Keep Cashiering ownership with requests from Collections, as the BRD-4 Collections FRS specifies; give Marketing read access to the items of its unit. Proposed behaviour: The Cashier assigns and the Cashiering TL approves; Collections asks through Incoming Requests (BRD-4). Available as a setting: Setting of what Marketing users see in the unapplied payment list: their marketing unit (BDOI's reading) by default.</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Add AP Unapplied Commission for reversed ORs; keep AR Insurer as a receivable, shown on the list for information. (the system reference FRS: AR Insurer is a receivable from the insurer set up by Adjustment; no AP Unapplied Commission.)</t>
+          <t>Add AP Unapplied Commission for reversed ORs; keep AR Insurer as a receivable, shown on the list for information. Proposed behaviour: AR Insurer is a receivable from the insurer set up by Adjustment; no AP Unapplied Commission.</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -4649,7 +4649,7 @@
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>Keep the the system warehouse (BRD); load it from the PMS list, so PMS stays the source of the checks. (the system reference FRS: Checks are warehoused in the system with a PDCW number and matured by the daily run (FR-OP-016).)</t>
+          <t>Keep the the system warehouse (BRD); load it from the PMS list, so PMS stays the source of the checks. Proposed behaviour: Checks are warehoused in the system with a PDCW number and matured by the daily run.</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
@@ -4685,7 +4685,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Adopt BDOI's forms. (the system reference FRS: The AR / OR PDF has a Cashier signature line; layout draft (this FRS).)</t>
+          <t>Adopt BDOI's forms. Proposed behaviour: The AR / OR PDF has a Cashier signature line; layout draft (this FRS).</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
@@ -4721,7 +4721,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Set 50 MB. (the system reference FRS: Not stated; the system accepts files up to 25 MB.) Available as a setting: Size limit per payment file type: 50 MB by default.</t>
+          <t>Set 50 MB. Proposed behaviour: Not stated; the system accepts files up to 25 MB. Available as a setting: Size limit per payment file type: 50 MB by default.</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>One rate from the Comptrollership table; reversals at the rate of the original receipt. (the system reference FRS: Comptrollership BOOK rate with 2 decimals at the receipt date; cancellation and reinstatement at the receipt's rate (FR-OP-027).)</t>
+          <t>One rate from the Comptrollership table; reversals at the rate of the original receipt. Proposed behaviour: Comptrollership BOOK rate with 2 decimals at the receipt date; cancellation and reinstatement at the receipt's rate.</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -4793,7 +4793,7 @@
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Keep the BRD list (it is a maintained list); add the check-payment restriction if BDOI wants it. (the system reference FRS: The BRD lists in four groups, including Check not picked-up, Negative VAT, Discount not applied, PDC retrieval / replacement, Bounced or returned check, Error printing.) Available as a setting: List of the cancellation reasons allowed for a check payment, by default.</t>
+          <t>Keep the BRD list (it is a maintained list); add the check-payment restriction if BDOI wants it. Proposed behaviour: The BRD lists in four groups, including Check not picked-up, Negative VAT, Discount not applied, PDC retrieval / replacement, Bounced or returned check, Error printing. Available as a setting: List of the cancellation reasons allowed for a check payment, by default.</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>By account, with the amount per account shown. (the system reference FRS: Partial reinstatement by amount.)</t>
+          <t>By account, with the amount per account shown. Proposed behaviour: Partial reinstatement by amount.</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
@@ -4865,7 +4865,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Keep them, defaulted from the receipt. (the system reference FRS: Invoice, AR / OR no., assured / payor, amount, Account Officer, Unit Head, Team Leader (premium); not required for a bounced check.)</t>
+          <t>Keep them, defaulted from the receipt. Proposed behaviour: Invoice, AR / OR no., assured / payor, amount, Account Officer, Unit Head, Team Leader (premium); not required for a bounced check.</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Enforce it through BDO's network and device policy if required; no change to the screens. (the system reference FRS: Log-in from a browser; responsive screens.) Available as a setting: Setting of the device restriction: off by default for SIT; on with the company networks and the device header of BDOI IT.</t>
+          <t>Enforce it through BDO's network and device policy if required; no change to the screens. Proposed behaviour: Log-in from a browser; responsive screens. Available as a setting: Setting of the device restriction: off by default for SIT; on with the company networks and the device header of BDOI IT.</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
@@ -4937,7 +4937,7 @@
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>Bank account mandatory (defaulted by currency as BDOI proposes); remarks optional. (the system reference FRS: Neither field exists on Receive Payment.) Available as a setting: Setting of the remarks of an AR: mandatory by default.</t>
+          <t>Bank account mandatory (defaulted by currency as BDOI proposes); remarks optional. Proposed behaviour: Neither field exists on Receive Payment. Available as a setting: Setting of the remarks of an AR: mandatory by default.</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -4973,7 +4973,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Tag per account, defaulted from the client; Comptrollership states the base of the 2% (basic or gross premium); the system keeps the share applied as a parameter. (the system reference FRS: 2% CWT client flag; 98% of the premium applied (FR-OP-018; OQ10).) Available as a setting: Setting of the base of the PR 2307: the premium amount by default; the basic premium available.</t>
+          <t>Tag per account, defaulted from the client; Comptrollership states the base of the 2% (basic or gross premium); the system keeps the share applied as a parameter. Proposed behaviour: 2% CWT client flag; 98% of the premium applied. Available as a setting: Setting of the base of the PR 2307: the premium amount by default; the basic premium available.</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
@@ -5009,7 +5009,7 @@
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>All applications, with a filter on the source (manual, file, PDC). (the system reference FRS: CSH-APPLIED-PREM lists every applied premium payment.)</t>
+          <t>All applications, with a filter on the source (manual, file, PDC). Proposed behaviour: CSH-APPLIED-PREM lists every applied premium payment.</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -5045,7 +5045,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Both documents propose the business uploads; record the change against the BRD (CLR-OP-08). (the system reference FRS: The Cashier uploads (FR-OP-015).)</t>
+          <t>Both documents propose the business uploads; record the change against the BRD. Proposed behaviour: The Cashier uploads.</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="D79" s="12" t="inlineStr">
         <is>
-          <t>Specify them in the FRS of Commission Receivables as BDOI maps them, or in the Marketing Collection and Disbursement FRS (BIBS FRS BRD-2 v2.1 FR-OP-113, FR-OP-121); Cashiering keeps the PR 2307 outstanding at payment (FRS.CSH.02.05.13).</t>
+          <t>Specify them in the FRS of Commission Receivables as BDOI maps them, or in the FRS of Marketing Collection and Disbursement; Cashiering keeps the PR 2307 outstanding at payment (FRS.CSH.02.05.13).</t>
         </is>
       </c>
       <c r="E79" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Operations Cashiering FRS v3.3 and classification rules v2 on both FRS: swimlane flows (shared flows/ generator), points beyond the BRD tested against the iNXT BrokerVerse OOTB platform (green) or change requests (orange, effort of the missing part), integration and data-migration scope labels, best-practice tables, Appendix W / Annex Y; effort workbooks with Summary, CR Effort, Beyond the BRD - OOTB, Integration & DM scope, Best practice, BRD items to deliver and Assumptions; BRD-02 builder reads the menu and message sheets of the retired sign-off workbook from a data file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'How to use'!$A$4:$D$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'How to use'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$27</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact assessment form'!$A$12:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Impact assessment form'!$12:$12</definedName>
@@ -796,7 +796,7 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>BRD-02 Operations Cashiering - after the sign-off of the FRS v3.2</t>
+          <t>BRD-02 Operations Cashiering - after the sign-off of the FRS v3.3</t>
         </is>
       </c>
     </row>
@@ -939,11 +939,11 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>Candidate changes known at v3.2 (status Candidate - for decision) and new requests</t>
+          <t>Candidate changes known at v3.3 (status Candidate - for decision) and new requests</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
-          <t>Row of Appendix R of the FRS v3.2</t>
+          <t>Row of Appendix R of the FRS v3.3</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr"/>
@@ -1913,7 +1913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T23"/>
+  <dimension ref="A1:T27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1948,7 +1948,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Candidate changes known at v3.2 (status Candidate - for decision) and new requests</t>
+          <t>Candidate changes known at v3.3 (status Candidate - for decision) and new requests</t>
         </is>
       </c>
     </row>
@@ -3710,29 +3710,369 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>CR-CSH-101</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Not in BRD</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Appendix J (time rules); FRS.CSH.02.05, FRS.CSH.03.01, FRS.CSH.04.01, FRS.CSH.06.02; FRS Appendix W.2</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Time rules of the Cashiering stages: overdue marker and reminder</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Records waiting for posting or approval are visible on the dashboard but nothing marks them late; a time rule per stage with a marker and a reminder keeps receipts issued the same day.</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Partial in BrokerVerse OOTB; the effort covers the missing part only: time rules, overdue marker and reminder for the Cashiering stages.</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved</t>
+        </is>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>6.5 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>BDOI to confirm the times (Appendix R, Appendix S)</t>
+        </is>
+      </c>
+      <c r="M24" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O24" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P24" s="12" t="inlineStr"/>
+      <c r="Q24" s="12" t="inlineStr"/>
+      <c r="R24" s="12" t="inlineStr"/>
+      <c r="S24" s="12" t="inlineStr"/>
+      <c r="T24" s="12" t="inlineStr">
+        <is>
+          <t>TC-OP-002.1-01, TC-OP-002.2-01, TC-OP-002.3-01, TC-OP-010.1-01, TC-OP-010.2-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>CR-CSH-102</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>BRQID.006 (extends)</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>FRS.CSH.10.03; Appendix G (failed batch run); FRS Appendix W.2</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>E-mail to a recipient list when a scheduled Cashiering run fails</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>The BRD asks that users are alerted when a run fails; an e-mail to named recipients makes sure a failed overnight run is seen before the business day starts.</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (e-mail to a recipient list).</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved</t>
+        </is>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>2.5 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>E-mail channel of BDOI</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O25" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P25" s="12" t="inlineStr"/>
+      <c r="Q25" s="12" t="inlineStr"/>
+      <c r="R25" s="12" t="inlineStr"/>
+      <c r="S25" s="12" t="inlineStr"/>
+      <c r="T25" s="12" t="inlineStr">
+        <is>
+          <t>TC-FRS-CSH.10.03.01-AC01, TC-FRS-CSH.10.03.01-AC02, TC-OP-008.1-01, TC-OP-008.2-01, TC-OP-008.3-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>CR-CSH-103</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>CSHID.023 (extends)</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>FRS.CSH.01.03.04; FRS Appendix W.2</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Excel export of the Cashiering lists</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Cashiers and Team Leaders work the lists in Excel for reconciliation and follow-up; the BRD asks for extracts of the reports, the FRS extends it to every list.</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="inlineStr">
+        <is>
+          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (Excel export of the lists).</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved</t>
+        </is>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>3 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L26" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M26" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O26" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P26" s="12" t="inlineStr"/>
+      <c r="Q26" s="12" t="inlineStr"/>
+      <c r="R26" s="12" t="inlineStr"/>
+      <c r="S26" s="12" t="inlineStr"/>
+      <c r="T26" s="12" t="inlineStr">
+        <is>
+          <t>TC-FRS-CSH.01.03.04-AC01, TC-FRS-CSH.01.03.04-AC02, TC-OP-003.4-01, TC-OP-003.1-01, TC-OP-003.2-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>CR-CSH-104</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Not in BRD</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>Appendix G (channel of each notice); FRS Appendix W.2</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Each user chooses an e-mail copy of the Cashiering notices</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Team Leaders who post from branches want the notices also by e-mail; the choice per user and per notice avoids e-mail floods.</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Beyond the BRD</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="inlineStr">
+        <is>
+          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (per-user, per-notice e-mail choice).</t>
+        </is>
+      </c>
+      <c r="J27" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved</t>
+        </is>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>3.5 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>E-mail channel of BDOI</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr">
+        <is>
+          <t>Test cases to add</t>
+        </is>
+      </c>
+      <c r="N27" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O27" s="25" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P27" s="12" t="inlineStr"/>
+      <c r="Q27" s="12" t="inlineStr"/>
+      <c r="R27" s="12" t="inlineStr"/>
+      <c r="S27" s="12" t="inlineStr"/>
+      <c r="T27" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:T23"/>
+  <autoFilter ref="A4:T27"/>
   <mergeCells count="1">
     <mergeCell ref="A2:T2"/>
   </mergeCells>
-  <conditionalFormatting sqref="O5:O523">
+  <conditionalFormatting sqref="O5:O527">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:T523">
+  <conditionalFormatting sqref="A5:T527">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H5:H523" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="H5:H527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N523" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="N5:N527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O523" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="O5:O527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$C$2:$C$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Product Maintenance v1.3 and Operations Cashiering v3.3: orange only where no BRD line covers the point (PM: 1 change request of 11.5 man-days; Cashiering: 2 of 10 man-days), BDOI FRS points covered by a BRD line listed as BRD points to deliver with planning effort, shared colours, workbook column Prepared for BIBS?, Programme README index of the current files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'How to use'!$A$4:$D$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'How to use'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Impact assessment form'!$A$12:$C$25</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Impact assessment form'!$12:$12</definedName>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23">
@@ -1913,7 +1913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T27"/>
+  <dimension ref="A1:T25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3814,22 +3814,22 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>BRQID.006 (extends)</t>
+          <t>Not in BRD</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>FRS.CSH.10.03; Appendix G (failed batch run); FRS Appendix W.2</t>
+          <t>Appendix G (channel of each notice); FRS Appendix W.2</t>
         </is>
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>E-mail to a recipient list when a scheduled Cashiering run fails</t>
+          <t>Each user chooses an e-mail copy of the Cashiering notices</t>
         </is>
       </c>
       <c r="G25" s="12" t="inlineStr">
         <is>
-          <t>The BRD asks that users are alerted when a run fails; an e-mail to named recipients makes sure a failed overnight run is seen before the business day starts.</t>
+          <t>Team Leaders who post from branches want the notices also by e-mail; the choice per user and per notice avoids e-mail floods.</t>
         </is>
       </c>
       <c r="H25" s="12" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (e-mail to a recipient list).</t>
+          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (per-user, per-notice e-mail choice).</t>
         </is>
       </c>
       <c r="J25" s="12" t="inlineStr">
@@ -3849,7 +3849,7 @@
       </c>
       <c r="K25" s="12" t="inlineStr">
         <is>
-          <t>2.5 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
+          <t>3.5 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
         </is>
       </c>
       <c r="L25" s="12" t="inlineStr">
@@ -3859,12 +3859,12 @@
       </c>
       <c r="M25" s="12" t="inlineStr">
         <is>
-          <t>Update the linked test cases</t>
+          <t>Test cases to add</t>
         </is>
       </c>
       <c r="N25" s="12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="O25" s="25" t="inlineStr">
@@ -3876,203 +3876,31 @@
       <c r="Q25" s="12" t="inlineStr"/>
       <c r="R25" s="12" t="inlineStr"/>
       <c r="S25" s="12" t="inlineStr"/>
-      <c r="T25" s="12" t="inlineStr">
-        <is>
-          <t>TC-FRS-CSH.10.03.01-AC01, TC-FRS-CSH.10.03.01-AC02, TC-OP-008.1-01, TC-OP-008.2-01, TC-OP-008.3-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="12" t="inlineStr">
-        <is>
-          <t>CR-CSH-103</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>11-Oct-2026</t>
-        </is>
-      </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>CSHID.023 (extends)</t>
-        </is>
-      </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>FRS.CSH.01.03.04; FRS Appendix W.2</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>Excel export of the Cashiering lists</t>
-        </is>
-      </c>
-      <c r="G26" s="12" t="inlineStr">
-        <is>
-          <t>Cashiers and Team Leaders work the lists in Excel for reconciliation and follow-up; the BRD asks for extracts of the reports, the FRS extends it to every list.</t>
-        </is>
-      </c>
-      <c r="H26" s="12" t="inlineStr">
-        <is>
-          <t>Beyond the BRD</t>
-        </is>
-      </c>
-      <c r="I26" s="12" t="inlineStr">
-        <is>
-          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (Excel export of the lists).</t>
-        </is>
-      </c>
-      <c r="J26" s="12" t="inlineStr">
-        <is>
-          <t>Within the drop if approved</t>
-        </is>
-      </c>
-      <c r="K26" s="12" t="inlineStr">
-        <is>
-          <t>3 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
-        </is>
-      </c>
-      <c r="L26" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M26" s="12" t="inlineStr">
-        <is>
-          <t>Update the linked test cases</t>
-        </is>
-      </c>
-      <c r="N26" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O26" s="25" t="inlineStr">
-        <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="P26" s="12" t="inlineStr"/>
-      <c r="Q26" s="12" t="inlineStr"/>
-      <c r="R26" s="12" t="inlineStr"/>
-      <c r="S26" s="12" t="inlineStr"/>
-      <c r="T26" s="12" t="inlineStr">
-        <is>
-          <t>TC-FRS-CSH.01.03.04-AC01, TC-FRS-CSH.01.03.04-AC02, TC-OP-003.4-01, TC-OP-003.1-01, TC-OP-003.2-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>CR-CSH-104</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>11-Oct-2026</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>iorta TechNXT Project Team</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Not in BRD</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
-        <is>
-          <t>Appendix G (channel of each notice); FRS Appendix W.2</t>
-        </is>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
-        <is>
-          <t>Each user chooses an e-mail copy of the Cashiering notices</t>
-        </is>
-      </c>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>Team Leaders who post from branches want the notices also by e-mail; the choice per user and per notice avoids e-mail floods.</t>
-        </is>
-      </c>
-      <c r="H27" s="12" t="inlineStr">
-        <is>
-          <t>Beyond the BRD</t>
-        </is>
-      </c>
-      <c r="I27" s="12" t="inlineStr">
-        <is>
-          <t>Partial in BrokerVerse OOTB; the effort is that of the missing part (per-user, per-notice e-mail choice).</t>
-        </is>
-      </c>
-      <c r="J27" s="12" t="inlineStr">
-        <is>
-          <t>Within the drop if approved</t>
-        </is>
-      </c>
-      <c r="K27" s="12" t="inlineStr">
-        <is>
-          <t>3.5 md (BIBS_CR_BRD-02_Effort_Estimate_v1.0.xlsx)</t>
-        </is>
-      </c>
-      <c r="L27" s="12" t="inlineStr">
-        <is>
-          <t>E-mail channel of BDOI</t>
-        </is>
-      </c>
-      <c r="M27" s="12" t="inlineStr">
-        <is>
-          <t>Test cases to add</t>
-        </is>
-      </c>
-      <c r="N27" s="12" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="O27" s="25" t="inlineStr">
-        <is>
-          <t>Candidate - for decision</t>
-        </is>
-      </c>
-      <c r="P27" s="12" t="inlineStr"/>
-      <c r="Q27" s="12" t="inlineStr"/>
-      <c r="R27" s="12" t="inlineStr"/>
-      <c r="S27" s="12" t="inlineStr"/>
-      <c r="T27" s="12" t="inlineStr"/>
+      <c r="T25" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:T27"/>
+  <autoFilter ref="A4:T25"/>
   <mergeCells count="1">
     <mergeCell ref="A2:T2"/>
   </mergeCells>
-  <conditionalFormatting sqref="O5:O527">
+  <conditionalFormatting sqref="O5:O525">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="1" stopIfTrue="1">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:T527">
+  <conditionalFormatting sqref="A5:T525">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="H5:H527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="H5:H525" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$5</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="N5:N525" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O527" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="O5:O525" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$C$2:$C$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
BDOI-template FRS packs: added content in BDOI's template styles, simulator wording replaced, one workbook style
- FRS (clean and highlighted, four packs): Arial throughout, body 10 pt, headings at BDOI's sizes per level,
  added tables 8 pt with the template's header fill, header words never broken, captions 9 pt italic,
  double spaces and empty paragraph runs removed, short notes kept with their table
- RTM test steps: test accounts / test files of BDOI's systems provided under the Integration scope
- Workbooks: file name and page in header/footer, print set-up, frozen and filtered header rows, man-days 0.00,
  costs #,##0.00, DayRate/Accuracy names on every effort estimate; BRD-03 inputs workbook in the common layout
- Programme index marks the Coverage and Comparison workbooks as internal

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-02_Operations_Cashiering/BIBS_CR_BRD-02_Change_Request_Register_v1.0.xlsx
@@ -1026,7 +1026,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1693,7 +1693,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -1906,7 +1906,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -3917,7 +3917,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -4232,7 +4232,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7353,7 +7353,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7516,7 +7516,7 @@
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
-    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
+    <oddHeader>&amp;L&amp;8 &amp;K004EA8Change Request Register&amp;C&amp;8 &amp;K656565&amp;F&amp;R&amp;8 &amp;K656565BDO Insure | BIBS – BDOI Broker System</oddHeader>
     <oddFooter>&amp;L&amp;8 &amp;K656565Confidential – BDOI&amp;C&amp;8 &amp;K656565Page &amp;P of &amp;N&amp;R&amp;8 &amp;K656565Version 1.0</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>